<commit_message>
Add CPT 93971 to Code Master
93971 is the unilateral/limited companion to 93970, which the workbook
already cross-referenced ("Use 93971 for unilateral or limited") without
listing the code itself.

- Insert 93971 on 'Code Master' row 22, in the US block directly after
  93970, with the official descriptor, the 'Venous duplex' category and a
  billing note pointing back to 93970 for a complete bilateral study.
- Extend the AutoFilter range to A4:F106 and keep the row styling, fill
  and heights of the US block.

The 'Specialties' counts are COUNTIF/COUNTIFS formulas over 'Code Master',
so Ultrasound now reads 6 codes and the total 102. Recalculated with no
formula errors.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014yTgcs7mEJWWAZRfzPEJGS
</commit_message>
<xml_diff>
--- a/Specialty_CPT_HCPCS_Code_Reference.xlsx
+++ b/Specialty_CPT_HCPCS_Code_Reference.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Notes &amp; Sources" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Code Master'!$A$4:$F$105</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Code Master'!$A$4:$F$106</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="370">
   <si>
     <t xml:space="preserve">Specialty Claims - CPT / HCPCS Code Reference</t>
   </si>
@@ -323,6 +323,15 @@
   </si>
   <si>
     <t xml:space="preserve">Complete bilateral. Use 93971 for unilateral or limited.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93971</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplex scan of extremity veins including responses to compression and other maneuvers; unilateral or limited study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unilateral or limited study. Use 93970 for a complete bilateral study.</t>
   </si>
   <si>
     <t xml:space="preserve">93978</t>
@@ -1360,16 +1369,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1409,11 +1422,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1469,7 +1482,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1817,174 +1830,174 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A5)</f>
         <v>4</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A5,'Code Master'!$C$5:$C$400,"CPT")</f>
         <v>4</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A5,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A6)</f>
         <v>9</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A6,'Code Master'!$C$5:$C$400,"CPT")</f>
         <v>9</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A6,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A7)</f>
-        <v>5</v>
-      </c>
-      <c r="E7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A7,'Code Master'!$C$5:$C$400,"CPT")</f>
-        <v>5</v>
-      </c>
-      <c r="F7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A7,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A8)</f>
         <v>39</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A8,'Code Master'!$C$5:$C$400,"CPT")</f>
         <v>39</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A8,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A9)</f>
         <v>44</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A9,'Code Master'!$C$5:$C$400,"CPT")</f>
         <v>1</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A9,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
         <v>43</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12"/>
-      <c r="B10" s="13" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="14" t="n">
+      <c r="C10" s="13"/>
+      <c r="D10" s="15" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>101</v>
-      </c>
-      <c r="E10" s="14" t="n">
+        <v>102</v>
+      </c>
+      <c r="E10" s="15" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>58</v>
-      </c>
-      <c r="F10" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="F10" s="15" t="n">
         <f aca="false">SUM(F5:F9)</f>
         <v>43</v>
       </c>
@@ -2005,2039 +2018,2059 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="C6" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="C7" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="C8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="6" t="s">
+      <c r="C10" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="C12" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+    <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="C14" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="C15" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="6" t="s">
+      <c r="C16" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="C17" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="6" t="s">
+      <c r="C18" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
+    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="C19" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="7" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="6" t="s">
+      <c r="C20" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="7" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="C22" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="F22" s="6" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" s="17" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
+      <c r="C23" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="F23" s="6" t="s">
+      <c r="B24" s="17" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
+      <c r="C24" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F24" s="6" t="s">
+      <c r="B25" s="17" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="C25" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="F25" s="6" t="s">
+      <c r="B26" s="17" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
+      <c r="C26" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="F26" s="6" t="s">
+      <c r="B27" s="17" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
+      <c r="C27" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B28" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
+      <c r="E28" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
+      <c r="B29" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="F29" s="6" t="s">
+      <c r="B30" s="17" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
+      <c r="C30" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="16" t="s">
+      <c r="B31" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="s">
+      <c r="E31" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
+      <c r="B32" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B32" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
+      <c r="B33" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B34" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="19" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
+      <c r="B36" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="19" t="s">
+      <c r="B37" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
+      <c r="B38" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B37" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="19" t="s">
+      <c r="B39" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="s">
+      <c r="B40" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E39" s="6" t="s">
+      <c r="B41" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="F39" s="6"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="19" t="s">
+      <c r="E41" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="F41" s="7"/>
+    </row>
+    <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="F40" s="6"/>
-    </row>
-    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="19" t="s">
+      <c r="B42" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B41" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="19" t="s">
+      <c r="B43" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B42" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="s">
+      <c r="B44" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F44" s="7"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B43" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F43" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="s">
+      <c r="B45" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="F45" s="7"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B44" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="F44" s="6"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="19" t="s">
+      <c r="B46" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="F46" s="7"/>
+    </row>
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="F45" s="6"/>
-    </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="19" t="s">
+      <c r="B47" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="F47" s="7"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="F46" s="6"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="19" t="s">
+      <c r="B48" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="F48" s="7"/>
+    </row>
+    <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B47" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E47" s="6" t="s">
+      <c r="B49" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="F47" s="6"/>
-    </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="19" t="s">
+      <c r="E49" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="s">
+      <c r="B50" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B49" s="16" t="s">
-        <v>173</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="19" t="s">
+      <c r="B51" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B52" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="C50" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="19" t="s">
+      <c r="E52" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B51" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="19" t="s">
+      <c r="B53" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B52" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="F52" s="6"/>
-    </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="19" t="s">
+      <c r="B54" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="F54" s="7"/>
+    </row>
+    <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="E53" s="6" t="s">
+      <c r="B55" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="F53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="19" t="s">
+      <c r="E55" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B54" s="16" t="s">
-        <v>187</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="19" t="s">
+      <c r="B56" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B55" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="19" t="s">
+      <c r="B57" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B56" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="F56" s="6"/>
-    </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="19" t="s">
+      <c r="B58" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B57" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E57" s="6" t="s">
+      <c r="B59" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D59" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="F57" s="6"/>
-    </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="19" t="s">
+      <c r="E59" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B58" s="16" t="s">
-        <v>199</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="F58" s="6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="19" t="s">
+      <c r="B60" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B59" s="16" t="s">
-        <v>202</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="F59" s="6" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="19" t="s">
+      <c r="B61" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="B60" s="16" t="s">
-        <v>206</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="F60" s="6" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B61" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="F61" s="6"/>
-    </row>
-    <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B62" s="21" t="s">
+      <c r="B62" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="C62" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D62" s="23" t="s">
+      <c r="C62" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E62" s="24" t="s">
+      <c r="E62" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="F62" s="25" t="s">
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B63" s="22" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B63" s="16" t="s">
+      <c r="C63" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="C63" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D63" s="6" t="s">
+      <c r="E63" s="25" t="s">
         <v>217</v>
       </c>
-      <c r="E63" s="6" t="s">
+      <c r="F63" s="26" t="s">
         <v>218</v>
       </c>
-      <c r="F63" s="6" t="s">
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64" s="17" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B64" s="16" t="s">
+      <c r="C64" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="C64" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="E64" s="6" t="s">
+      <c r="E64" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="F64" s="6" t="s">
+      <c r="F64" s="7" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B65" s="16" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B65" s="17" t="s">
         <v>223</v>
       </c>
-      <c r="C65" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="E65" s="6" t="s">
+      <c r="C65" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E65" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="F65" s="6" t="s">
+      <c r="F65" s="7" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B66" s="16" t="s">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B66" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="C66" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" s="6" t="s">
+      <c r="C66" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E66" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E66" s="6" t="s">
+      <c r="F66" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="F66" s="6" t="s">
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B67" s="17" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B67" s="16" t="s">
+      <c r="C67" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="C67" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="E67" s="6" t="s">
+      <c r="E67" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="F67" s="6" t="s">
+      <c r="F67" s="7" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B68" s="16" t="s">
+    <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" s="17" t="s">
         <v>233</v>
       </c>
-      <c r="C68" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68" s="6" t="s">
+      <c r="C68" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E68" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="F68" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="F68" s="6" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B69" s="16" t="s">
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B69" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="C69" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="E69" s="6" t="s">
+      <c r="C69" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="F69" s="6" t="s">
+      <c r="E69" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F69" s="7" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B70" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D70" s="6" t="s">
+    <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B70" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="C70" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E70" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="F70" s="6" t="s">
+      <c r="F70" s="7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B71" s="17" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B71" s="16" t="s">
+      <c r="C71" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="C71" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D71" s="6" t="s">
+      <c r="E71" s="7" t="s">
         <v>243</v>
       </c>
-      <c r="E71" s="6" t="s">
+      <c r="F71" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="F71" s="6" t="s">
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B72" s="17" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B72" s="16" t="s">
+      <c r="C72" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="C72" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="E72" s="6" t="s">
+      <c r="E72" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="F72" s="6"/>
-    </row>
-    <row r="73" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B73" s="16" t="s">
+      <c r="F72" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="C73" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D73" s="6" t="s">
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B73" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="E73" s="6" t="s">
+      <c r="C73" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="E73" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="F73" s="6" t="s">
+      <c r="F73" s="7"/>
+    </row>
+    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B74" s="17" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B74" s="16" t="s">
+      <c r="C74" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="C74" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="E74" s="6" t="s">
+      <c r="E74" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="F74" s="6" t="s">
+      <c r="F74" s="7" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B75" s="16" t="s">
+    <row r="75" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B75" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="C75" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="6" t="s">
+      <c r="C75" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="E75" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="E75" s="6" t="s">
+      <c r="F75" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="F75" s="6" t="s">
+    </row>
+    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B76" s="17" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="76" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B76" s="16" t="s">
+      <c r="C76" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="C76" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D76" s="6" t="s">
+      <c r="E76" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="E76" s="6" t="s">
+      <c r="F76" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="F76" s="6" t="s">
+    </row>
+    <row r="77" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B77" s="17" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="77" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B77" s="16" t="s">
+      <c r="C77" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="C77" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="6" t="s">
+      <c r="E77" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="E77" s="6" t="s">
+      <c r="F77" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="F77" s="6" t="s">
+    </row>
+    <row r="78" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B78" s="17" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="78" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B78" s="16" t="s">
+      <c r="C78" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="C78" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="E78" s="6" t="s">
+      <c r="E78" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="F78" s="6" t="s">
+      <c r="F78" s="7" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B79" s="16" t="s">
+    <row r="79" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B79" s="17" t="s">
         <v>270</v>
       </c>
-      <c r="C79" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D79" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="E79" s="6" t="s">
+      <c r="C79" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="E79" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="F79" s="6" t="s">
+      <c r="F79" s="7" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B80" s="16" t="s">
+    <row r="80" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B80" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D80" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="E80" s="6" t="s">
+      <c r="C80" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="E80" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="F80" s="6" t="s">
+      <c r="F80" s="7" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B81" s="16" t="s">
+    <row r="81" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B81" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="C81" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D81" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="E81" s="6" t="s">
+      <c r="C81" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="E81" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="F81" s="6" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B82" s="16" t="s">
+      <c r="F81" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="C82" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D82" s="6" t="s">
+    </row>
+    <row r="82" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B82" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="C82" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="E82" s="7" t="s">
         <v>280</v>
       </c>
-      <c r="F82" s="6"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B83" s="16" t="s">
+      <c r="F82" s="7" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B83" s="17" t="s">
         <v>281</v>
       </c>
-      <c r="C83" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D83" s="6" t="s">
+      <c r="C83" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" s="7" t="s">
         <v>282</v>
       </c>
-      <c r="E83" s="6" t="s">
+      <c r="E83" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="F83" s="6" t="s">
+      <c r="F83" s="7"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B84" s="17" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="84" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B84" s="16" t="s">
+      <c r="C84" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="7" t="s">
         <v>285</v>
       </c>
-      <c r="C84" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D84" s="6" t="s">
+      <c r="E84" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="E84" s="6" t="s">
+      <c r="F84" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="F84" s="6" t="s">
+    </row>
+    <row r="85" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B85" s="17" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="85" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B85" s="16" t="s">
+      <c r="C85" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="C85" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D85" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="E85" s="6" t="s">
+      <c r="E85" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="F85" s="6" t="s">
+      <c r="F85" s="7" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B86" s="16" t="s">
+    <row r="86" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B86" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="C86" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="E86" s="6" t="s">
+      <c r="C86" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E86" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="F86" s="6" t="s">
+      <c r="F86" s="7" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B87" s="16" t="s">
+    <row r="87" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B87" s="17" t="s">
         <v>295</v>
       </c>
-      <c r="C87" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="E87" s="6" t="s">
+      <c r="C87" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E87" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="F87" s="6" t="s">
+      <c r="F87" s="7" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B88" s="16" t="s">
+    <row r="88" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B88" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="C88" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D88" s="6" t="s">
-        <v>286</v>
-      </c>
-      <c r="E88" s="6" t="s">
+      <c r="C88" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E88" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="F88" s="6" t="s">
+      <c r="F88" s="7" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B89" s="16" t="s">
+    <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B89" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="C89" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D89" s="6" t="s">
+      <c r="C89" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E89" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="E89" s="6" t="s">
+      <c r="F89" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="F89" s="6" t="s">
+    </row>
+    <row r="90" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B90" s="17" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B90" s="16" t="s">
+      <c r="C90" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="C90" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D90" s="6" t="s">
-        <v>302</v>
-      </c>
-      <c r="E90" s="6" t="s">
+      <c r="E90" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="F90" s="6" t="s">
+      <c r="F90" s="7" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B91" s="16" t="s">
+    <row r="91" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B91" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="C91" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="6" t="s">
+      <c r="C91" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="E91" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="E91" s="6" t="s">
+      <c r="F91" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="F91" s="6" t="s">
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B92" s="17" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B92" s="16" t="s">
+      <c r="C92" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D92" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="C92" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D92" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E92" s="6" t="s">
+      <c r="E92" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="F92" s="6" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B93" s="16" t="s">
+      <c r="F92" s="7" t="s">
         <v>314</v>
       </c>
-      <c r="C93" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D93" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E93" s="6" t="s">
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B93" s="17" t="s">
         <v>315</v>
       </c>
-      <c r="F93" s="6" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B94" s="16" t="s">
+      <c r="C93" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E93" s="7" t="s">
         <v>316</v>
       </c>
-      <c r="C94" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D94" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E94" s="6" t="s">
+      <c r="F93" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B94" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="F94" s="6" t="s">
+      <c r="C94" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E94" s="7" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B95" s="16" t="s">
+      <c r="F94" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B95" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="C95" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D95" s="6" t="s">
+      <c r="C95" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E95" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="E95" s="6" t="s">
+      <c r="F95" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="F95" s="6" t="s">
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B96" s="17" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B96" s="16" t="s">
+      <c r="C96" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="7" t="s">
         <v>323</v>
       </c>
-      <c r="C96" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D96" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="E96" s="6" t="s">
+      <c r="E96" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="F96" s="6" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B97" s="16" t="s">
+      <c r="F96" s="7" t="s">
         <v>325</v>
       </c>
-      <c r="C97" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="E97" s="6" t="s">
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B97" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="F97" s="6" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B98" s="16" t="s">
+      <c r="C97" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E97" s="7" t="s">
         <v>327</v>
       </c>
-      <c r="C98" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D98" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E98" s="6" t="s">
+      <c r="F97" s="7" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B98" s="17" t="s">
         <v>328</v>
       </c>
-      <c r="F98" s="6" t="s">
+      <c r="C98" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E98" s="7" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B99" s="16" t="s">
+      <c r="F98" s="7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B99" s="17" t="s">
         <v>330</v>
       </c>
-      <c r="C99" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D99" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E99" s="6" t="s">
+      <c r="C99" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E99" s="7" t="s">
         <v>331</v>
       </c>
-      <c r="F99" s="6" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B100" s="16" t="s">
+      <c r="F99" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="C100" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D100" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E100" s="6" t="s">
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B100" s="17" t="s">
         <v>333</v>
       </c>
-      <c r="F100" s="6" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B101" s="16" t="s">
+      <c r="C100" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E100" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="C101" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D101" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="E101" s="6" t="s">
+      <c r="F100" s="7" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B101" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="F101" s="6" t="s">
+      <c r="C101" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E101" s="7" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B102" s="16" t="s">
+      <c r="F101" s="7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B102" s="17" t="s">
         <v>337</v>
       </c>
-      <c r="C102" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D102" s="6" t="s">
+      <c r="C102" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E102" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="E102" s="6" t="s">
+      <c r="F102" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="F102" s="6" t="s">
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B103" s="17" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="103" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B103" s="21" t="s">
+      <c r="C103" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D103" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="C103" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="D103" s="23" t="s">
-        <v>338</v>
-      </c>
-      <c r="E103" s="24" t="s">
+      <c r="E103" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="F103" s="25" t="s">
+      <c r="F103" s="7" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B104" s="16" t="s">
+    <row r="104" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B104" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="C104" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D104" s="6" t="s">
+      <c r="C104" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D104" s="24" t="s">
+        <v>341</v>
+      </c>
+      <c r="E104" s="25" t="s">
         <v>345</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="F104" s="26" t="s">
         <v>346</v>
       </c>
-      <c r="F104" s="6" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B105" s="16" t="s">
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B105" s="17" t="s">
         <v>347</v>
       </c>
-      <c r="C105" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D105" s="6" t="s">
+      <c r="C105" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="E105" s="6" t="s">
+      <c r="E105" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="F105" s="6" t="s">
-        <v>258</v>
+      <c r="F105" s="7" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B106" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E106" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="F106" s="7" t="s">
+        <v>261</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F105"/>
+  <autoFilter ref="A4:F106"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4058,107 +4091,107 @@
   <dimension ref="A1:A23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="128"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="128"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>351</v>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="28" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>352</v>
+      <c r="A4" s="29" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
-        <v>353</v>
+      <c r="A5" s="29" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="s">
-        <v>355</v>
+      <c r="A6" s="29" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="29"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
-        <v>356</v>
+      <c r="A9" s="29" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27" t="s">
-        <v>358</v>
+      <c r="A10" s="29" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="29"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="s">
-        <v>360</v>
+      <c r="A13" s="29" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="29"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="28" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
-        <v>362</v>
+      <c r="A16" s="29" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="29"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
-        <v>363</v>
+      <c r="A19" s="29" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
-        <v>364</v>
+      <c r="A20" s="29" t="s">
+        <v>367</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
+      <c r="A21" s="29" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="29"/>
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
-        <v>366</v>
+      <c r="A23" s="29" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add CPT 93922 to Code Master
93922 is the limited (1-2 level) counterpart to 93923, which the workbook
already listed for studies at 3 or more levels.

- Insert 93922 on 'Code Master' row 19, in the US block directly above
  93923, with the official descriptor, the 'Physiologic arterial study'
  category and a billing note covering the level threshold and the
  modifier 52 requirement for a unilateral study.
- Extend the AutoFilter range to A4:F107; the row is left on auto-fit so
  the long descriptor is sized to its content.

Ultrasound now reads 7 codes and the total 103. Recalculated with no
formula errors.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014yTgcs7mEJWWAZRfzPEJGS
</commit_message>
<xml_diff>
--- a/Specialty_CPT_HCPCS_Code_Reference.xlsx
+++ b/Specialty_CPT_HCPCS_Code_Reference.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Notes &amp; Sources" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Code Master'!$A$4:$F$106</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Code Master'!$A$4:$F$107</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="373">
   <si>
     <t xml:space="preserve">Specialty Claims - CPT / HCPCS Code Reference</t>
   </si>
@@ -289,10 +289,19 @@
     <t xml:space="preserve">Carotid/vertebral duplex, complete bilateral.</t>
   </si>
   <si>
+    <t xml:space="preserve">93922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physiologic arterial study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limited bilateral noninvasive physiologic studies of upper or lower extremity arteries, (eg, for lower extremity: ankle/brachial indices at distal posterior tibial and anterior tibial/dorsalis pedis arteries plus bidirectional, Doppler waveform recording and analysis, at 1-2 levels, or ankle/brachial indices at distal posterior tibial and anterior tibial/dorsalis pedis arteries plus volume plethysmography at 1-2 levels, or ankle/brachial indices at distal posterior tibial and anterior tibial/dorsalis pedis arteries with, transcutaneous oxygen tension measurements at 1-2 levels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limited bilateral study, 1-2 levels. Use 93923 for 3 or more levels. Append modifier 52 for a unilateral study.</t>
+  </si>
+  <si>
     <t xml:space="preserve">93923</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Physiologic arterial study</t>
   </si>
   <si>
     <t xml:space="preserve">Complete bilateral noninvasive physiologic studies of upper or lower extremity arteries, 3 or more levels (eg, for lower extremity: ankle/brachial indices at distal posterior tibial and anterior tibial/dorsalis pedis arteries plus segmental blood pressure measurements), or single level study with provocative functional maneuvers</t>
@@ -1926,11 +1935,11 @@
       </c>
       <c r="D7" s="8" t="n">
         <f aca="false">COUNTIF('Code Master'!$A$5:$A$400,$A7)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A7,'Code Master'!$C$5:$C$400,"CPT")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">COUNTIFS('Code Master'!$A$5:$A$400,$A7,'Code Master'!$C$5:$C$400,"HCPCS Level II")</f>
@@ -1991,11 +2000,11 @@
       <c r="C10" s="13"/>
       <c r="D10" s="15" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E10" s="15" t="n">
         <f aca="false">SUM(E5:E9)</f>
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F10" s="15" t="n">
         <f aca="false">SUM(F5:F9)</f>
@@ -2018,7 +2027,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -2339,7 +2348,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
         <v>14</v>
       </c>
@@ -2359,7 +2368,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
         <v>14</v>
       </c>
@@ -2370,13 +2379,13 @@
         <v>6</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2384,19 +2393,19 @@
         <v>14</v>
       </c>
       <c r="B21" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2404,13 +2413,13 @@
         <v>14</v>
       </c>
       <c r="B22" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>89</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>93</v>
@@ -2430,33 +2439,33 @@
         <v>6</v>
       </c>
       <c r="D23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="F23" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="7" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B24" s="17" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="17" t="s">
+      <c r="C24" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="E24" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="F24" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2464,73 +2473,73 @@
         <v>17</v>
       </c>
       <c r="B25" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C25" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="7" t="s">
+      <c r="E26" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="F27" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B28" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>112</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>116</v>
@@ -2550,7 +2559,7 @@
         <v>6</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>119</v>
@@ -2570,33 +2579,33 @@
         <v>6</v>
       </c>
       <c r="D30" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="F30" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>125</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>126</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2604,19 +2613,19 @@
         <v>17</v>
       </c>
       <c r="B32" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2630,73 +2639,73 @@
         <v>6</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>131</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>134</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>137</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>140</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2704,13 +2713,13 @@
         <v>17</v>
       </c>
       <c r="B37" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>143</v>
@@ -2730,32 +2739,34 @@
         <v>6</v>
       </c>
       <c r="D38" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E38" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="F38" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="F38" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B39" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C39" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" s="7" t="s">
+      <c r="E39" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="E39" s="7" t="s">
+      <c r="F39" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="F39" s="7"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
@@ -2768,10 +2779,10 @@
         <v>6</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F40" s="7"/>
     </row>
@@ -2780,38 +2791,36 @@
         <v>17</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F41" s="7"/>
     </row>
-    <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="F42" s="7" t="s">
         <v>158</v>
       </c>
+      <c r="F42" s="7"/>
     </row>
     <row r="43" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="20" t="s">
@@ -2824,7 +2833,7 @@
         <v>6</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>160</v>
@@ -2833,7 +2842,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="20" t="s">
         <v>17</v>
       </c>
@@ -2844,28 +2853,30 @@
         <v>6</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="F44" s="7"/>
+      <c r="F44" s="7" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F45" s="7"/>
     </row>
@@ -2874,31 +2885,31 @@
         <v>17</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F46" s="7"/>
     </row>
-    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="E47" s="7" t="s">
         <v>170</v>
@@ -2916,10 +2927,10 @@
         <v>6</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F48" s="7"/>
     </row>
@@ -2928,20 +2939,18 @@
         <v>17</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="F49" s="7" t="s">
         <v>175</v>
       </c>
+      <c r="F49" s="7"/>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="s">
@@ -2954,13 +2963,13 @@
         <v>6</v>
       </c>
       <c r="D50" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="E50" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="E50" s="7" t="s">
+      <c r="F50" s="7" t="s">
         <v>178</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2968,19 +2977,19 @@
         <v>17</v>
       </c>
       <c r="B51" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D51" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="E51" s="7" t="s">
         <v>181</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2988,19 +2997,19 @@
         <v>17</v>
       </c>
       <c r="B52" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F52" s="7" t="s">
         <v>182</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3014,12 +3023,14 @@
         <v>6</v>
       </c>
       <c r="D53" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E53" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="E53" s="7" t="s">
+      <c r="F53" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="F53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="20" t="s">
@@ -3032,10 +3043,10 @@
         <v>6</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F54" s="7"/>
     </row>
@@ -3044,20 +3055,18 @@
         <v>17</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="F55" s="7" t="s">
         <v>192</v>
       </c>
+      <c r="F55" s="7"/>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="20" t="s">
@@ -3070,13 +3079,13 @@
         <v>6</v>
       </c>
       <c r="D56" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E56" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E56" s="7" t="s">
+      <c r="F56" s="7" t="s">
         <v>195</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3084,18 +3093,20 @@
         <v>17</v>
       </c>
       <c r="B57" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C57" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D57" s="7" t="s">
+      <c r="E57" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="E57" s="7" t="s">
+      <c r="F57" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="F57" s="7"/>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="20" t="s">
@@ -3108,10 +3119,10 @@
         <v>6</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F58" s="7"/>
     </row>
@@ -3120,22 +3131,20 @@
         <v>17</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E59" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="F59" s="7" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="20" t="s">
         <v>17</v>
       </c>
@@ -3146,27 +3155,27 @@
         <v>6</v>
       </c>
       <c r="D60" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="E60" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="E60" s="7" t="s">
+      <c r="F60" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="F60" s="7" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B61" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D61" s="7" t="s">
         <v>209</v>
-      </c>
-      <c r="C61" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>206</v>
       </c>
       <c r="E61" s="7" t="s">
         <v>210</v>
@@ -3175,7 +3184,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="20" t="s">
         <v>17</v>
       </c>
@@ -3186,51 +3195,51 @@
         <v>6</v>
       </c>
       <c r="D62" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E62" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E62" s="7" t="s">
+      <c r="F62" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="F62" s="7"/>
-    </row>
-    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B63" s="22" t="s">
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" s="17" t="s">
         <v>215</v>
       </c>
-      <c r="C63" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D63" s="24" t="s">
+      <c r="C63" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E63" s="25" t="s">
+      <c r="E63" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="F63" s="26" t="s">
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B64" s="22" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B64" s="17" t="s">
+      <c r="C64" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D64" s="24" t="s">
         <v>219</v>
       </c>
-      <c r="C64" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64" s="7" t="s">
+      <c r="E64" s="25" t="s">
         <v>220</v>
       </c>
-      <c r="E64" s="7" t="s">
+      <c r="F64" s="26" t="s">
         <v>221</v>
-      </c>
-      <c r="F64" s="7" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3238,13 +3247,13 @@
         <v>20</v>
       </c>
       <c r="B65" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="C65" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>224</v>
@@ -3264,7 +3273,7 @@
         <v>7</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>227</v>
@@ -3284,27 +3293,27 @@
         <v>7</v>
       </c>
       <c r="D67" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E67" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="E67" s="7" t="s">
+      <c r="F67" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="F67" s="7" t="s">
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B68" s="17" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B68" s="17" t="s">
+      <c r="C68" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="7" t="s">
         <v>233</v>
-      </c>
-      <c r="C68" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>230</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>234</v>
@@ -3313,7 +3322,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="27" t="s">
         <v>20</v>
       </c>
@@ -3324,16 +3333,16 @@
         <v>7</v>
       </c>
       <c r="D69" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E69" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="E69" s="7" t="s">
+      <c r="F69" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="F69" s="7" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="27" t="s">
         <v>20</v>
       </c>
@@ -3344,33 +3353,33 @@
         <v>7</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="27" t="s">
         <v>20</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>243</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3378,19 +3387,19 @@
         <v>20</v>
       </c>
       <c r="B72" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="C72" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="7" t="s">
+      <c r="E72" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="E72" s="7" t="s">
+      <c r="F72" s="7" t="s">
         <v>247</v>
-      </c>
-      <c r="F72" s="7" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3398,51 +3407,51 @@
         <v>20</v>
       </c>
       <c r="B73" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="7" t="s">
         <v>249</v>
-      </c>
-      <c r="C73" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>246</v>
       </c>
       <c r="E73" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="F73" s="7"/>
-    </row>
-    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F73" s="7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="27" t="s">
         <v>20</v>
       </c>
       <c r="B74" s="17" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="F74" s="7" t="s">
+      <c r="F74" s="7"/>
+    </row>
+    <row r="75" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B75" s="17" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="75" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B75" s="17" t="s">
+      <c r="C75" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="7" t="s">
         <v>255</v>
-      </c>
-      <c r="C75" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>252</v>
       </c>
       <c r="E75" s="7" t="s">
         <v>256</v>
@@ -3451,7 +3460,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="27" t="s">
         <v>20</v>
       </c>
@@ -3462,33 +3471,33 @@
         <v>7</v>
       </c>
       <c r="D76" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="E76" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="F76" s="7" t="s">
         <v>260</v>
       </c>
-      <c r="F76" s="7" t="s">
+    </row>
+    <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B77" s="17" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="77" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B77" s="17" t="s">
+      <c r="C77" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="C77" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="7" t="s">
+      <c r="E77" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="E77" s="7" t="s">
+      <c r="F77" s="7" t="s">
         <v>264</v>
-      </c>
-      <c r="F77" s="7" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3496,33 +3505,33 @@
         <v>20</v>
       </c>
       <c r="B78" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="C78" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" s="7" t="s">
+      <c r="E78" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="E78" s="7" t="s">
+      <c r="F78" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="F78" s="7" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B79" s="17" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="79" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B79" s="17" t="s">
+      <c r="C79" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79" s="7" t="s">
         <v>270</v>
-      </c>
-      <c r="C79" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D79" s="7" t="s">
-        <v>263</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>271</v>
@@ -3542,7 +3551,7 @@
         <v>7</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E80" s="7" t="s">
         <v>274</v>
@@ -3551,7 +3560,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="27" t="s">
         <v>20</v>
       </c>
@@ -3562,7 +3571,7 @@
         <v>7</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E81" s="7" t="s">
         <v>277</v>
@@ -3582,32 +3591,34 @@
         <v>7</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E82" s="7" t="s">
         <v>280</v>
       </c>
       <c r="F82" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="27" t="s">
         <v>20</v>
       </c>
       <c r="B83" s="17" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="F83" s="7"/>
+      <c r="F83" s="7" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="27" t="s">
@@ -3625,28 +3636,26 @@
       <c r="E84" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="F84" s="7" t="s">
+      <c r="F84" s="7"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B85" s="17" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="85" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B85" s="17" t="s">
+      <c r="C85" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" s="7" t="s">
         <v>288</v>
       </c>
-      <c r="C85" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D85" s="7" t="s">
+      <c r="E85" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="E85" s="7" t="s">
+      <c r="F85" s="7" t="s">
         <v>290</v>
-      </c>
-      <c r="F85" s="7" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3654,13 +3663,13 @@
         <v>20</v>
       </c>
       <c r="B86" s="17" t="s">
+        <v>291</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="7" t="s">
         <v>292</v>
-      </c>
-      <c r="C86" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" s="7" t="s">
-        <v>289</v>
       </c>
       <c r="E86" s="7" t="s">
         <v>293</v>
@@ -3669,7 +3678,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="27" t="s">
         <v>20</v>
       </c>
@@ -3680,7 +3689,7 @@
         <v>7</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>296</v>
@@ -3700,7 +3709,7 @@
         <v>7</v>
       </c>
       <c r="D88" s="7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>299</v>
@@ -3720,7 +3729,7 @@
         <v>7</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>302</v>
@@ -3740,13 +3749,13 @@
         <v>7</v>
       </c>
       <c r="D90" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="E90" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="E90" s="7" t="s">
+      <c r="F90" s="7" t="s">
         <v>306</v>
-      </c>
-      <c r="F90" s="7" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3754,13 +3763,13 @@
         <v>20</v>
       </c>
       <c r="B91" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="7" t="s">
         <v>308</v>
-      </c>
-      <c r="C91" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="7" t="s">
-        <v>305</v>
       </c>
       <c r="E91" s="7" t="s">
         <v>309</v>
@@ -3769,7 +3778,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="27" t="s">
         <v>20</v>
       </c>
@@ -3780,13 +3789,13 @@
         <v>7</v>
       </c>
       <c r="D92" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="E92" s="7" t="s">
         <v>312</v>
       </c>
-      <c r="E92" s="7" t="s">
+      <c r="F92" s="7" t="s">
         <v>313</v>
-      </c>
-      <c r="F92" s="7" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3794,19 +3803,19 @@
         <v>20</v>
       </c>
       <c r="B93" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" s="7" t="s">
         <v>315</v>
-      </c>
-      <c r="C93" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D93" s="7" t="s">
-        <v>312</v>
       </c>
       <c r="E93" s="7" t="s">
         <v>316</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3814,19 +3823,19 @@
         <v>20</v>
       </c>
       <c r="B94" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="F94" s="7" t="s">
         <v>317</v>
-      </c>
-      <c r="C94" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="E94" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="F94" s="7" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3834,19 +3843,19 @@
         <v>20</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3860,13 +3869,13 @@
         <v>7</v>
       </c>
       <c r="D96" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="E96" s="7" t="s">
         <v>323</v>
       </c>
-      <c r="E96" s="7" t="s">
+      <c r="F96" s="7" t="s">
         <v>324</v>
-      </c>
-      <c r="F96" s="7" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3874,19 +3883,19 @@
         <v>20</v>
       </c>
       <c r="B97" s="17" t="s">
+        <v>325</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D97" s="7" t="s">
         <v>326</v>
-      </c>
-      <c r="C97" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D97" s="7" t="s">
-        <v>323</v>
       </c>
       <c r="E97" s="7" t="s">
         <v>327</v>
       </c>
       <c r="F97" s="7" t="s">
-        <v>314</v>
+        <v>328</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3894,42 +3903,42 @@
         <v>20</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C98" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F98" s="7" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="27" t="s">
         <v>20</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C99" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F99" s="7" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="27" t="s">
         <v>20</v>
       </c>
@@ -3940,13 +3949,13 @@
         <v>7</v>
       </c>
       <c r="D100" s="7" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E100" s="7" t="s">
         <v>334</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3954,19 +3963,19 @@
         <v>20</v>
       </c>
       <c r="B101" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F101" s="7" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3974,19 +3983,19 @@
         <v>20</v>
       </c>
       <c r="B102" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F102" s="7" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4000,56 +4009,56 @@
         <v>7</v>
       </c>
       <c r="D103" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="E103" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="E103" s="7" t="s">
+      <c r="F103" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="F103" s="7" t="s">
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B104" s="17" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="104" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B104" s="22" t="s">
+      <c r="C104" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D104" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="C104" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D104" s="24" t="s">
-        <v>341</v>
-      </c>
-      <c r="E104" s="25" t="s">
+      <c r="E104" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="F104" s="26" t="s">
+      <c r="F104" s="7" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="B105" s="17" t="s">
+    <row r="105" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B105" s="22" t="s">
         <v>347</v>
       </c>
-      <c r="C105" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D105" s="7" t="s">
+      <c r="C105" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105" s="24" t="s">
+        <v>344</v>
+      </c>
+      <c r="E105" s="25" t="s">
         <v>348</v>
       </c>
-      <c r="E105" s="7" t="s">
+      <c r="F105" s="26" t="s">
         <v>349</v>
       </c>
-      <c r="F105" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="27" t="s">
         <v>20</v>
       </c>
@@ -4066,11 +4075,31 @@
         <v>352</v>
       </c>
       <c r="F106" s="7" t="s">
-        <v>261</v>
+        <v>264</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B107" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="E107" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="F107" s="7" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F106"/>
+  <autoFilter ref="A4:F107"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4096,27 +4125,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4124,17 +4153,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="29" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="29" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4142,12 +4171,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4155,12 +4184,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="29" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4168,22 +4197,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="29" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="29" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4191,7 +4220,7 @@
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="29" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>